<commit_message>
Stock à jour : ajout de 2 attaches QCS60 en colonne S60
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Lesstocks.xlsx
+++ b/Lesstocks.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Desktop\Mes applis\Machines\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51C14C83-ED81-4BA6-9B37-1ACC6859EB8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3F35D43-CC1A-46E8-86BA-E30F0409C0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{58AB1E1A-7D1F-4F7D-8D28-6E6C076A80FB}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="43">
   <si>
     <t>DIAM65</t>
   </si>
@@ -154,6 +154,9 @@
   </si>
   <si>
     <t>BRH HB32</t>
+  </si>
+  <si>
+    <t>Attache QCS60</t>
   </si>
 </sst>
 </file>
@@ -659,6 +662,9 @@
       <c r="C6" s="1" t="s">
         <v>41</v>
       </c>
+      <c r="F6" s="1" t="s">
+        <v>42</v>
+      </c>
       <c r="H6" s="3" t="s">
         <v>36</v>
       </c>
@@ -669,6 +675,9 @@
       </c>
       <c r="B7" t="s">
         <v>20</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>42</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
Champ 'Nom du client' par pelle (renseigné à la vente), sauvegardé et inclus dans l'export/import JSON
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Lesstocks.xlsx
+++ b/Lesstocks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Desktop\Mes applis\Machines\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3F35D43-CC1A-46E8-86BA-E30F0409C0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B95819A-B582-41B5-AEB7-148EE120CBF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{58AB1E1A-7D1F-4F7D-8D28-6E6C076A80FB}"/>
+    <workbookView xWindow="7125" yWindow="5535" windowWidth="28800" windowHeight="15345" xr2:uid="{58AB1E1A-7D1F-4F7D-8D28-6E6C076A80FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="66">
   <si>
     <t>DIAM65</t>
   </si>
@@ -157,6 +157,75 @@
   </si>
   <si>
     <t>Attache QCS60</t>
+  </si>
+  <si>
+    <t>Adaptateur a souder platine</t>
+  </si>
+  <si>
+    <t>Attache QC70</t>
+  </si>
+  <si>
+    <t>Tilt X18</t>
+  </si>
+  <si>
+    <t>Tilt X26</t>
+  </si>
+  <si>
+    <t>Arrivage fouille 1400  300</t>
+  </si>
+  <si>
+    <t>Arrivage attache UA63 350</t>
+  </si>
+  <si>
+    <t>Arrivage fouille 1500  350</t>
+  </si>
+  <si>
+    <t>Arrivage platine HB32</t>
+  </si>
+  <si>
+    <t>Arrivage Petit dx100</t>
+  </si>
+  <si>
+    <t>Arrivage Moyen dx100</t>
+  </si>
+  <si>
+    <t>Arrivage Curage dx100</t>
+  </si>
+  <si>
+    <t>Arrivage Platine hb08</t>
+  </si>
+  <si>
+    <t>Arrivage Attache UA23</t>
+  </si>
+  <si>
+    <t>Arrivage attache UA 53 210</t>
+  </si>
+  <si>
+    <t>Arrivage fouille 1200</t>
+  </si>
+  <si>
+    <t>Arrivage squelette  1200</t>
+  </si>
+  <si>
+    <t>Arrivage platine HB22</t>
+  </si>
+  <si>
+    <t>Arrivage Curage 2000</t>
+  </si>
+  <si>
+    <t>Arrivage Fouille 600</t>
+  </si>
+  <si>
+    <t>Arrivage attache UA53</t>
+  </si>
+  <si>
+    <t>Arrivage attache UA63 360</t>
+  </si>
+  <si>
+    <t>Arrivage fouille 1500  360</t>
+  </si>
+  <si>
+    <t>Arrivage platine libre</t>
   </si>
 </sst>
 </file>
@@ -534,7 +603,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{489AD73F-0A86-4110-B7A7-D1612688A31A}">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="8" width="30.7109375" customWidth="1"/>
@@ -648,6 +717,9 @@
       <c r="F5" t="s">
         <v>31</v>
       </c>
+      <c r="G5" t="s">
+        <v>43</v>
+      </c>
       <c r="H5" s="3" t="s">
         <v>36</v>
       </c>
@@ -665,6 +737,9 @@
       <c r="F6" s="1" t="s">
         <v>42</v>
       </c>
+      <c r="G6" s="1" t="s">
+        <v>44</v>
+      </c>
       <c r="H6" s="3" t="s">
         <v>36</v>
       </c>
@@ -676,8 +751,14 @@
       <c r="B7" t="s">
         <v>20</v>
       </c>
+      <c r="C7" s="1" t="s">
+        <v>47</v>
+      </c>
       <c r="F7" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>36</v>
@@ -690,6 +771,12 @@
       <c r="B8" t="s">
         <v>23</v>
       </c>
+      <c r="C8" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="H8" s="3" t="s">
         <v>37</v>
       </c>
@@ -701,49 +788,64 @@
       <c r="B9" t="s">
         <v>23</v>
       </c>
+      <c r="C9" s="1" t="s">
+        <v>48</v>
+      </c>
       <c r="H9" s="3" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>12</v>
+      <c r="A10" t="s">
+        <v>11</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>21</v>
       </c>
+      <c r="C10" s="1" t="s">
+        <v>48</v>
+      </c>
       <c r="H10" s="3" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>13</v>
+      <c r="A11" s="1" t="s">
+        <v>12</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="C11" s="1" t="s">
+        <v>49</v>
+      </c>
       <c r="H11" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>12</v>
+      <c r="A12" t="s">
+        <v>13</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="C12" s="1" t="s">
+        <v>49</v>
+      </c>
       <c r="H12" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>40</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>38</v>
@@ -753,13 +855,25 @@
       <c r="A14" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="B14" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>50</v>
+      </c>
       <c r="H14" s="3" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>39</v>
@@ -767,55 +881,188 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="B18" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="B19" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+      <c r="B20" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="B21" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B22" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>19</v>
+      </c>
+      <c r="B25" t="s">
+        <v>60</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B27" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H28" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H29" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H30" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H31" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H32" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="33" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H33" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="34" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H34" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="35" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H35" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="36" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H36" s="3" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>